<commit_message>
Build P01 reporting controls, decimal engine, mapping and verified exports
</commit_message>
<xml_diff>
--- a/examples/Apex_Horizon_Technologies_Inc._Financial_Statements_FY2025.xlsx
+++ b/examples/Apex_Horizon_Technologies_Inc._Financial_Statements_FY2025.xlsx
@@ -3,12 +3,13 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Trial Balance" sheetId="1" r:id="rId1"/>
-    <sheet name="Profit and Loss" sheetId="2" r:id="rId2"/>
-    <sheet name="Financial Position" sheetId="3" r:id="rId3"/>
-    <sheet name="Changes in Equity" sheetId="4" r:id="rId4"/>
-    <sheet name="Cash Flows" sheetId="5" r:id="rId5"/>
-    <sheet name="Ratios" sheetId="6" r:id="rId6"/>
+    <sheet name="Validation" sheetId="1" r:id="rId1"/>
+    <sheet name="Trial Balance" sheetId="2" r:id="rId2"/>
+    <sheet name="Profit and Loss" sheetId="3" r:id="rId3"/>
+    <sheet name="Financial Position" sheetId="4" r:id="rId4"/>
+    <sheet name="Changes in Equity" sheetId="5" r:id="rId5"/>
+    <sheet name="Cash Flows" sheetId="6" r:id="rId6"/>
+    <sheet name="Ratios" sheetId="7" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -402,6 +403,123 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D8"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="B1" t="str">
+        <v>DRAFT - mathematical checks only; no compliance certification</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Control</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Result</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Difference</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Explanation</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Debit = Credit</v>
+      </c>
+      <c r="B3" t="str">
+        <v>pass</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3" t="str">
+        <v>20 mapped accounts. Difference must be exactly zero.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Account signs</v>
+      </c>
+      <c r="B4" t="str">
+        <v>pass</v>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v>2 contra accounts. Debit and credit signs are preserved; contra accounts are not flipped twice.</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Financial position</v>
+      </c>
+      <c r="B5" t="str">
+        <v>pass</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Assets must equal liabilities plus equity, including current-period profit once.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Opening equity</v>
+      </c>
+      <c r="B6" t="str">
+        <v>pass</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Opening total is compared with prior-period closing equity. Component allocation still needs review.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Equity movements</v>
+      </c>
+      <c r="B7" t="str">
+        <v>pass</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Opening equity + profit + capital issued − dividends + OCI must equal closing equity. Movements must already be posted to the ledger.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Cash flow inputs</v>
+      </c>
+      <c r="B8" t="str">
+        <v>pass</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Comparative data and movements reconcile to closing cash. Review classifications before use.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D8"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H26"/>
   <sheetData>
     <row r="1">
@@ -989,7 +1107,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B26"/>
   <sheetData>
@@ -1184,7 +1302,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B40"/>
   <sheetData>
@@ -1467,9 +1585,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:E10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1498,6 +1616,9 @@
         <v>Retained Earnings</v>
       </c>
       <c r="D4" t="str">
+        <v>Other Reserves</v>
+      </c>
+      <c r="E4" t="str">
         <v>Total Equity</v>
       </c>
     </row>
@@ -1512,6 +1633,9 @@
         <v>82000</v>
       </c>
       <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
         <v>182000</v>
       </c>
     </row>
@@ -1526,6 +1650,9 @@
         <v>35000</v>
       </c>
       <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
         <v>35000</v>
       </c>
     </row>
@@ -1542,10 +1669,13 @@
       <c r="D7">
         <v>0</v>
       </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Dividends Paid</v>
+        <v>Dividends Declared</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -1554,59 +1684,54 @@
         <v>-5000</v>
       </c>
       <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
         <v>-5000</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Opening other reserves</v>
-      </c>
-      <c r="B9" t="str">
-        <v/>
-      </c>
-      <c r="C9" t="str">
-        <v/>
+        <v>Other comprehensive income</v>
+      </c>
+      <c r="B9">
+        <v>0</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
       </c>
       <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9">
         <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Other comprehensive income</v>
-      </c>
-      <c r="B10" t="str">
-        <v/>
-      </c>
-      <c r="C10" t="str">
-        <v/>
+        <v>Closing Balance</v>
+      </c>
+      <c r="B10">
+        <v>100000</v>
+      </c>
+      <c r="C10">
+        <v>112000</v>
       </c>
       <c r="D10">
         <v>0</v>
       </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>Closing Balance</v>
-      </c>
-      <c r="B11">
-        <v>100000</v>
-      </c>
-      <c r="C11">
-        <v>112000</v>
-      </c>
-      <c r="D11">
+      <c r="E10">
         <v>212000</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E10"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B34"/>
   <sheetData>
@@ -1857,7 +1982,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G14"/>
   <sheetData>

</xml_diff>